<commit_message>
Update Nikkei225 Ver7 research data
</commit_message>
<xml_diff>
--- a/reports/daily/nikkei225_ranking_ver7_20260818.xlsx
+++ b/reports/daily/nikkei225_ranking_ver7_20260818.xlsx
@@ -707,7 +707,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SUMITOMO MITSUI TRUST GP INC</t>
+          <t>三井住友トラストグループ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -860,7 +860,7 @@
         <v>1734</v>
       </c>
       <c r="AV2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -896,7 +896,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SUZUKI MOTOR CORP</t>
+          <t>スズキ</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1045,7 +1045,7 @@
         <v>2081</v>
       </c>
       <c r="AV3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW3" t="n">
         <v>0</v>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NOMURA HOLDINGS INC.</t>
+          <t>野村ホールディングス</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1230,7 +1230,7 @@
         <v>1554</v>
       </c>
       <c r="AV4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW4" t="n">
         <v>0</v>
@@ -1266,7 +1266,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DAIICHI LIFE GROUP INC</t>
+          <t>第一生命ホールディングス</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1419,7 +1419,7 @@
         <v>1841.5</v>
       </c>
       <c r="AV5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DAIWA SECURITIES GROUP</t>
+          <t>大和証券グループ本社</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1604,7 +1604,7 @@
         <v>1771</v>
       </c>
       <c r="AV6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW6" t="n">
         <v>0</v>
@@ -1640,7 +1640,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YOKOHAMA RUBBER CO</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1789,7 +1789,7 @@
         <v>7647</v>
       </c>
       <c r="AV7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW7" t="n">
         <v>0</v>
@@ -1825,7 +1825,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LY CORPORATION</t>
+          <t>LINEヤフー</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1974,7 +1974,7 @@
         <v>497.9</v>
       </c>
       <c r="AV8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW8" t="n">
         <v>0</v>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DIC CORPORATION</t>
+          <t>DIC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2159,7 +2159,7 @@
         <v>5495</v>
       </c>
       <c r="AV9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW9" t="n">
         <v>0</v>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MIZUHO FINANCIAL GROUP</t>
+          <t>みずほフィナンシャルグループ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2348,7 +2348,7 @@
         <v>8531</v>
       </c>
       <c r="AV10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW10" t="n">
         <v>0</v>
@@ -2384,7 +2384,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">MITSUBISHI UFJ FINANCIAL GROUP </t>
+          <t>三菱UFJフィナンシャル・グループ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2537,7 +2537,7 @@
         <v>3654</v>
       </c>
       <c r="AV11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW11" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CHIBA BANK</t>
+          <t>千葉銀行</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2722,7 +2722,7 @@
         <v>2837.5</v>
       </c>
       <c r="AV12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW12" t="n">
         <v>0</v>
@@ -2758,7 +2758,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MS&amp;AD INS GP HLDGS</t>
+          <t>MS&amp;ADインシュアランスグループホールディングス</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2907,7 +2907,7 @@
         <v>4985</v>
       </c>
       <c r="AV13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW13" t="n">
         <v>0</v>
@@ -2943,7 +2943,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KIRIN HOLDINGS COMPANY LIMITED</t>
+          <t>キリンホールディングス</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -3092,7 +3092,7 @@
         <v>3000</v>
       </c>
       <c r="AV14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW14" t="n">
         <v>0</v>
@@ -3128,7 +3128,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BRIDGESTONE CORP</t>
+          <t>ブリヂストン</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3277,7 +3277,7 @@
         <v>4074</v>
       </c>
       <c r="AV15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW15" t="n">
         <v>0</v>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NISSAN CHEMICAL CORPORATION</t>
+          <t>日産化学</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3462,7 +3462,7 @@
         <v>8059</v>
       </c>
       <c r="AV16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW16" t="n">
         <v>0</v>
@@ -3498,7 +3498,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IDEMITSU KOSAN CO.LTD</t>
+          <t>出光興産</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3647,7 +3647,7 @@
         <v>1370.5</v>
       </c>
       <c r="AV17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW17" t="n">
         <v>0</v>
@@ -3683,7 +3683,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OTSUKA HLDGS CO LTD</t>
+          <t>大塚ホールディングス</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -3832,7 +3832,7 @@
         <v>12040</v>
       </c>
       <c r="AV18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW18" t="n">
         <v>0</v>
@@ -3868,7 +3868,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SUMITOMO MITSUI FINANCIAL GROUP</t>
+          <t>三井住友フィナンシャルグループ</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -4021,7 +4021,7 @@
         <v>6900</v>
       </c>
       <c r="AV19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW19" t="n">
         <v>0</v>
@@ -4057,7 +4057,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NICHIREI CORP</t>
+          <t>ニチレイ</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -4206,7 +4206,7 @@
         <v>2141.5</v>
       </c>
       <c r="AV20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW20" t="n">
         <v>0</v>
@@ -4242,7 +4242,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>FUKUOKA FINANCIAL GROUP INC.</t>
+          <t>ふくおかフィナンシャルグループ</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -4409,7 +4409,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ORIX CORPORATION</t>
+          <t>オリックス</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ASTELLAS PHARMA</t>
+          <t>アステラス製薬</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4747,7 +4747,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>OKUMA CORPORATION</t>
+          <t>オークマ</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -4914,7 +4914,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ADVANTEST CORP</t>
+          <t>アドバンテスト</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>AJINOMOTO CO INC</t>
+          <t>味の素</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -5252,7 +5252,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>KIKKOMAN CORP</t>
+          <t>キッコーマン</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>RESONA HOLDINGS</t>
+          <t>りそなホールディングス</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>JAPAN TOBACCO INC</t>
+          <t>日本たばこ産業（JT）</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5761,7 +5761,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>NITTO DENKO CORP</t>
+          <t>日東電工</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -5932,7 +5932,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>DOWA HOLDINGS</t>
+          <t>DOWAホールディングス</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>T&amp;D HOLDINGS INC</t>
+          <t>T&amp;Dホールディングス</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -6266,7 +6266,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>TERUMO CORP</t>
+          <t>テルモ</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>KYOCERA CORP</t>
+          <t>京セラ</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -6600,7 +6600,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ANA HOLDINGS INC</t>
+          <t>ANAホールディングス</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -6767,7 +6767,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>HITACHI CONSTRUCTION MACHINERY</t>
+          <t>日立建機</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>JAPAN POST HLDGS CO LTD</t>
+          <t>日本郵政</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -7101,7 +7101,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KEISEI ELECTRIC RAILWAY CO</t>
+          <t>京成電鉄</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -7268,7 +7268,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SEIKO EPSON CORP</t>
+          <t>セイコーエプソン</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -7439,7 +7439,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SUMITOMO HEAVY INDUSTRIES</t>
+          <t>住友重機械工業</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -7606,7 +7606,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>KYOWA KIRIN CO LTD</t>
+          <t>協和キリン</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CANON INC</t>
+          <t>キヤノン</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>KOMATSU</t>
+          <t>小松製作所</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>KONAMI GROUP CORPORATION</t>
+          <t>コナミグループ</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>JAPAN AIRLINES CO LTD</t>
+          <t>日本航空</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -8441,7 +8441,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MATSUI SECURITIES CO</t>
+          <t>松井証券</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -8606,7 +8606,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CREDIT SAISON CO</t>
+          <t>クレディセゾン</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -8773,7 +8773,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>NTT INC</t>
+          <t>NTT</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -8944,7 +8944,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>YAMAHA CORP</t>
+          <t>ヤマハ</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -9111,7 +9111,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TOYOTA TSUSHO CORP</t>
+          <t>豊田通商</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -9278,7 +9278,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>NISSUI CORPORATION</t>
+          <t>ニッスイ</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -9445,7 +9445,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>NIPPON EXPRESS HLDGS INC</t>
+          <t>NIPPON EXPRESSホールディングス</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -9612,7 +9612,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TOKAI CARBON CO</t>
+          <t>東海カーボン</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -9779,7 +9779,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MITSUI CHEMICALS INC</t>
+          <t>三井化学</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -9946,7 +9946,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>YOKOHAMA FINANCIAL GROUP INC</t>
+          <t>コンコルディア・フィナンシャルグループ</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -10111,7 +10111,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TORAY INDUSTRIES INC</t>
+          <t>東レ</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -10278,7 +10278,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>RICOH CO</t>
+          <t>リコー</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -10445,7 +10445,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>SUMITOMO METAL MINING CO</t>
+          <t>住友金属鉱山</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -10612,7 +10612,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>SUMITOMO CORP</t>
+          <t>住友商事</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -10779,7 +10779,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>KAO CORP</t>
+          <t>花王</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -10946,7 +10946,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>CITIZEN WATCH CO LTD</t>
+          <t>シチズン時計</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -11113,7 +11113,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ENEOS HOLDINGS INC</t>
+          <t>ENEOSホールディングス</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -11278,7 +11278,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>HONDA MOTOR CO</t>
+          <t>本田技研工業</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -11443,7 +11443,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>PANASONIC HOLDINGS CORP</t>
+          <t>パナソニック ホールディングス</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -11610,7 +11610,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SONY GROUP CORPORATION</t>
+          <t>ソニーグループ</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -11781,7 +11781,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SUMITOMO OSAKA CEMENT CO</t>
+          <t>住友大阪セメント</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -11944,7 +11944,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>KURARAY CO</t>
+          <t>クラレ</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -12111,7 +12111,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>KDDI CORPORATION</t>
+          <t>KDDI</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -12282,7 +12282,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MITSUBISHI CHEMICAL GROUP CORP</t>
+          <t>三菱ケミカルグループ</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -12447,7 +12447,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>OMRON CORP</t>
+          <t>オムロン</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>FUJI ELECTRIC CO. LTD.</t>
+          <t>富士電機</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -12785,7 +12785,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>BANDAI NAMCO HOLDINGS INC</t>
+          <t>バンダイナムコホールディングス</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -12952,7 +12952,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>RECRUIT HOLDINGS CO LTD</t>
+          <t>リクルートホールディングス</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -13119,7 +13119,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>HOYA CORP</t>
+          <t>HOYA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -13286,7 +13286,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>KEYENCE CORP</t>
+          <t>キーエンス</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -13455,7 +13455,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>IHI CORPORATION</t>
+          <t>IHI</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -13491,7 +13491,7 @@
         <v>5.2</v>
       </c>
       <c r="K76" t="n">
-        <v>4.9</v>
+        <v>4.5</v>
       </c>
       <c r="L76" t="n">
         <v>33.4</v>
@@ -13622,7 +13622,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>NIPPON YUSEN KABUSHIKI KAISHA</t>
+          <t>日本郵船</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -13789,7 +13789,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>UBE CORPORATION</t>
+          <t>UBE</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -13956,7 +13956,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>TOYOTA MOTOR CORP</t>
+          <t>トヨタ自動車</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -14123,7 +14123,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>NIDEC CORPORATION</t>
+          <t>ニデック</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -14294,7 +14294,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>UNITIKA LTD</t>
+          <t>ユニチカ</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -14459,7 +14459,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SOFTBANK CORP.</t>
+          <t>ソフトバンク</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -14630,7 +14630,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>TOBU RAILWAY CO</t>
+          <t>東武鉄道</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -14797,7 +14797,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>TOPPAN HOLDINGS INC</t>
+          <t>TOPPANホールディングス</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -14964,7 +14964,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>KANSAI ELECTRIC POWER CO INC</t>
+          <t>関西電力</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -15131,7 +15131,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>DAI NIPPON PRINTING CO</t>
+          <t>大日本印刷</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -15298,7 +15298,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>JTEKT CORPORATION</t>
+          <t>ジェイテクト</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>MITSUI O.S.K. LINES LTD</t>
+          <t>商船三井</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -15632,7 +15632,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>RESONAC HOLDINGS CORPORATION</t>
+          <t>レゾナック・ホールディングス</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -15799,7 +15799,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>TAIHEIYO CEMENT CORP</t>
+          <t>太平洋セメント</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -15966,7 +15966,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>JFE HOLDINGS INC</t>
+          <t>JFEホールディングス</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -16133,7 +16133,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>SAPPORO BREWERIES LTD</t>
+          <t>サッポロホールディングス</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -16298,7 +16298,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>ITOCHU CORP</t>
+          <t>伊藤忠商事</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -16469,7 +16469,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>EISAI CO LTD</t>
+          <t>エーザイ</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -16636,7 +16636,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MITSUBISHI MATERIALS CORP</t>
+          <t>三菱マテリアル</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -16801,7 +16801,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>SHISEIDO COMPANY LIMITED</t>
+          <t>資生堂</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -16966,7 +16966,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>MITSUBISHI CORP</t>
+          <t>三菱商事</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -17137,7 +17137,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>TAKASHIMAYA CO</t>
+          <t>高島屋</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -17302,7 +17302,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MAZDA MOTOR CORP</t>
+          <t>マツダ</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -17467,7 +17467,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>INPEX CORPORATION</t>
+          <t>INPEX</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -17634,7 +17634,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>HASEKO CORPORATION</t>
+          <t>長谷工コーポレーション</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -17801,7 +17801,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>TDK CORP</t>
+          <t>TDK</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -17968,7 +17968,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>OLYMPUS CORPORATION</t>
+          <t>オリンパス</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -18135,7 +18135,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>COMSYS HOLDINGS CORP</t>
+          <t>コムシスホールディングス</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -18302,7 +18302,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>FUJIKURA</t>
+          <t>フジクラ</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -18465,7 +18465,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>SEKISUI HOUSE</t>
+          <t>積水ハウス</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -18632,7 +18632,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>NIPPON STEEL CORPORATION</t>
+          <t>日本製鉄</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -18797,7 +18797,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>KAWASAKI HEAVY INDUSTRIES</t>
+          <t>川崎重工業</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -18964,7 +18964,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>KOBE STEEL</t>
+          <t>神戸製鋼所</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -19127,7 +19127,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>MITSUBISHI LOGISTICS CORP</t>
+          <t>三菱倉庫</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -19294,7 +19294,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>DAIWA HOUSE INDUSTRY CO</t>
+          <t>大和ハウス工業</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -19461,7 +19461,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>OJI HOLDINGS CORP</t>
+          <t>王子ホールディングス</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -19626,7 +19626,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>MEIJI HOLDINGS CO LTD</t>
+          <t>明治ホールディングス</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -19793,7 +19793,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>KUBOTA CORP</t>
+          <t>クボタ</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -19960,7 +19960,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>SHIONOGI &amp; CO</t>
+          <t>塩野義製薬</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -20127,7 +20127,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>TOKYO TATEMONO CO</t>
+          <t>東京建物</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -20294,7 +20294,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>TOYOBO CO</t>
+          <t>東洋紡</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -20461,7 +20461,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>NTN CORP</t>
+          <t>NTN</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -20628,7 +20628,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>NEC CORP</t>
+          <t>NEC</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -20799,7 +20799,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>CENTRAL JAPAN RAILWAY CO</t>
+          <t>JR東海</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -20966,7 +20966,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>SUMITOMO CHEMICAL COMPANY</t>
+          <t>住友化学</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -21131,7 +21131,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>FURUKAWA ELECTRIC CO</t>
+          <t>古河電気工業</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -21298,7 +21298,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>SOFTBANK GROUP CORP</t>
+          <t>ソフトバンクグループ</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -21469,7 +21469,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>MARUI GROUP CO LTD</t>
+          <t>丸井グループ</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -21636,7 +21636,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>KAWASAKI KISEN KAISHA</t>
+          <t>川崎汽船</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -21803,7 +21803,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>JGC HOLDINGS CORPORATION</t>
+          <t>日揮ホールディングス</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -21970,7 +21970,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>MITSUBISHI ELECTRIC CORP</t>
+          <t>三菱電機</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -22139,7 +22139,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>FAST RETAILING CO LTD</t>
+          <t>ファーストリテイリング</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -22306,7 +22306,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>ASAHI KASEI CORP</t>
+          <t>旭化成</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -22473,7 +22473,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>NSK</t>
+          <t>日本精工</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -22640,7 +22640,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>HITACHI</t>
+          <t>日立製作所</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>JAPAN EXCHANGE GROUP</t>
+          <t>日本取引所グループ</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -22970,7 +22970,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>RYOHIN KEIKAKU CO</t>
+          <t>良品計画</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -23135,7 +23135,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>TAKEDA PHARMACEUTICAL CO LTD</t>
+          <t>武田薬品工業</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -23300,7 +23300,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>CHUBU ELECTRIC POWER CO INC</t>
+          <t>中部電力</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -23467,7 +23467,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>ODAKYU ELECTRIC RAILWAY CO</t>
+          <t>小田急電鉄</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -23634,7 +23634,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>ALPS ALPINE CO LTD</t>
+          <t>アルプスアルパイン</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -23799,7 +23799,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>NISSHIN SEIFUN GROUP INC</t>
+          <t>日清製粉グループ本社</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -23966,7 +23966,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>ASAHI GROUP HLDGS</t>
+          <t>アサヒグループホールディングス</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -24133,7 +24133,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>SEVEN &amp; I HOLDINGS CO LTD</t>
+          <t>セブン＆アイ・ホールディングス</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -24300,7 +24300,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>MITSUI &amp; CO</t>
+          <t>三井物産</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -24471,7 +24471,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>TOKYO ELECTRON</t>
+          <t>東京エレクトロン</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -24642,7 +24642,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>NGK CORP</t>
+          <t>日本ガイシ</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -24809,7 +24809,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>NITORI HOLDINGS CO LTD</t>
+          <t>ニトリホールディングス</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -24976,7 +24976,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>MITSUBISHI HEAVY INDUSTRIES</t>
+          <t>三菱重工業</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -25143,7 +25143,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>KIOXIA HOLDINGS CORPORATION</t>
+          <t>キオクシアホールディングス</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -25310,7 +25310,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>NEXON CO LTD</t>
+          <t>ネクソン</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -25477,7 +25477,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>DENA CO LTD</t>
+          <t>ディー・エヌ・エー</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -25644,7 +25644,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>MURATA MANUFACTURING CO</t>
+          <t>村田製作所</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -25815,7 +25815,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>TEIJIN LTD</t>
+          <t>帝人</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -25978,7 +25978,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>KEIO CORPORATION</t>
+          <t>京王電鉄</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -26145,7 +26145,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>TOSOH CORP</t>
+          <t>東ソー</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -26310,7 +26310,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>RENESAS ELECTRONICS CORP</t>
+          <t>ルネサスエレクトロニクス</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -26479,7 +26479,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>SUMITOMO ELECTRIC INDUSTRIES</t>
+          <t>住友電気工業</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -26646,7 +26646,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>DAIICHI SANKYO COMPANY LIMITED</t>
+          <t>第一三共</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -26813,7 +26813,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>AMADA CO LTD</t>
+          <t>アマダ</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -26978,7 +26978,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>KANADEVIA CORPORATION</t>
+          <t>カナデビア</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -27141,7 +27141,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>PAN PACIFIC INTL HLDGS CORP</t>
+          <t>パン・パシフィック・インターナショナルホールディングス</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -27306,7 +27306,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>DENSO CORP</t>
+          <t>デンソー</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -27473,7 +27473,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>OBAYASHI CORP</t>
+          <t>大林組</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -27640,7 +27640,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>WEST JAPAN RAILWAY CO</t>
+          <t>JR西日本</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -27807,7 +27807,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>TOHO CO LTD</t>
+          <t>東宝</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -27974,7 +27974,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>SUMITOMO PHARMA CO LTD</t>
+          <t>住友ファーマ</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -28139,7 +28139,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>MARUBENI CORP</t>
+          <t>丸紅</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -28310,7 +28310,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>J FRONT RETAILING CO LTD</t>
+          <t>J.フロント リテイリング</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -28477,7 +28477,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>FUJITSU</t>
+          <t>富士通</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -28648,7 +28648,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>SHIMIZU CORP</t>
+          <t>清水建設</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -28815,7 +28815,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>ISUZU MOTORS</t>
+          <t>いすゞ自動車</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -28982,7 +28982,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>ISETAN MITSUKOSHI HOLDINGS LTD</t>
+          <t>三越伊勢丹ホールディングス</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -29147,7 +29147,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>EBARA CORP</t>
+          <t>荏原製作所</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -29314,7 +29314,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>NH FOODS LTD</t>
+          <t>日本ハム</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -29481,7 +29481,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>ZOZO INC</t>
+          <t>ZOZO</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -29648,7 +29648,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>SHIN-ETSU CHEMICAL CO</t>
+          <t>信越化学工業</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -29819,7 +29819,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>MITSUBISHI MOTOR CORP</t>
+          <t>三菱自動車工業</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -29986,7 +29986,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>TOKYU FUDOSAN HOLDINGS CORPORAT</t>
+          <t>東急不動産ホールディングス</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -30153,7 +30153,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>DENTSU GROUP INC</t>
+          <t>電通グループ</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -30310,7 +30310,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>SUMCO CORPORATION</t>
+          <t>SUMCO</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -30473,7 +30473,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>CHUGAI PHARMACEUTICAL CO</t>
+          <t>中外製薬</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -30640,7 +30640,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>TOKYO GAS CO</t>
+          <t>東京ガス</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -30807,7 +30807,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>SUBARU CORPORATION</t>
+          <t>SUBARU</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -30974,7 +30974,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>SCREEN HOLDINGS CO LTD</t>
+          <t>SCREENホールディングス</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -31141,7 +31141,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>NINTENDO CO LTD</t>
+          <t>任天堂</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -31306,7 +31306,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>YAMATO HOLDINGS CO LTD</t>
+          <t>ヤマトホールディングス</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -31471,7 +31471,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>SECOM CO</t>
+          <t>セコム</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -31638,7 +31638,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>AGC INC</t>
+          <t>AGC</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -31803,7 +31803,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>MITSUBISHI ESTATE CO</t>
+          <t>三菱地所</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -31970,7 +31970,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>TOKIO MARINE HOLDINGS INC</t>
+          <t>東京海上ホールディングス</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -32139,7 +32139,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>M3 INC</t>
+          <t>エムスリー</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -32300,7 +32300,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>OSAKA GAS CO</t>
+          <t>大阪ガス</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -32467,7 +32467,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>TOKYO METRO CO LTD</t>
+          <t>東京地下鉄</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -32632,7 +32632,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>YOKOGAWA ELECTRIC CORP</t>
+          <t>横河電機</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -32797,7 +32797,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>SHARP CORP</t>
+          <t>シャープ</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -32962,7 +32962,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>TOKYU CORP</t>
+          <t>東急</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -33127,7 +33127,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>TAIYO YUDEN CO LTD</t>
+          <t>太陽誘電</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -33292,7 +33292,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>AEON CO LTD</t>
+          <t>イオン</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -33457,7 +33457,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>DAIKIN INDUSTRIES</t>
+          <t>ダイキン工業</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -33620,7 +33620,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>TOKYO ELEC POWER CO HLDGS INC</t>
+          <t>東京電力ホールディングス</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -33781,7 +33781,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>DENKA COMPANY LIMITED</t>
+          <t>デンカ</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -33944,7 +33944,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>EAST JAPAN RAILWAY CO</t>
+          <t>JR東日本</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -34111,7 +34111,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>NIKON CORP</t>
+          <t>ニコン</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -34276,7 +34276,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>TAISEI CORP</t>
+          <t>大成建設</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -34441,7 +34441,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>CYBER AGENT</t>
+          <t>サイバーエージェント</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -34608,7 +34608,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>MITSUI FUDOSAN</t>
+          <t>三井不動産</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -34775,7 +34775,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>MITSUI KINZOKU CO LTD</t>
+          <t>三井金属</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -34940,7 +34940,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>LASERTEC CORP</t>
+          <t>レーザーテック</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -34976,7 +34976,7 @@
         <v>33.9</v>
       </c>
       <c r="K205" t="n">
-        <v>14.7</v>
+        <v>13.4</v>
       </c>
       <c r="L205" t="n">
         <v>33.9</v>
@@ -35107,7 +35107,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>TOTO LTD</t>
+          <t>TOTO</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -35274,7 +35274,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>FUJIFILM HOLDINGS CORPORATION</t>
+          <t>富士フイルムホールディングス</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -35441,7 +35441,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>TREND MICRO INC</t>
+          <t>トレンドマイクロ</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -35608,7 +35608,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>SUMITOMO REALTY &amp; DEVELOPMENT C</t>
+          <t>住友不動産</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -35771,7 +35771,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>FANUC CORPORATION</t>
+          <t>ファナック</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -35938,7 +35938,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>KAJIMA CORP</t>
+          <t>鹿島建設</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -36103,7 +36103,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>NISSAN MOTOR CO</t>
+          <t>日産自動車</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -36264,7 +36264,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>TOKUYAMA CORP</t>
+          <t>トクヤマ</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -36425,7 +36425,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>NIPPON ELECTRIC GLASS</t>
+          <t>日本電気硝子</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -36590,7 +36590,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>RAKUTEN GROUP INC</t>
+          <t>楽天グループ</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -36751,7 +36751,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>YASKAWA ELECTRIC CORP</t>
+          <t>安川電機</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -36918,7 +36918,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>SOCIONEXT INC</t>
+          <t>ソシオネクスト</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -37374,7 +37374,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SUMITOMO MITSUI TRUST GP INC</t>
+          <t>三井住友トラストグループ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -37527,7 +37527,7 @@
         <v>1734</v>
       </c>
       <c r="AV2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -37563,7 +37563,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SUZUKI MOTOR CORP</t>
+          <t>スズキ</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -37712,7 +37712,7 @@
         <v>2081</v>
       </c>
       <c r="AV3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW3" t="n">
         <v>0</v>
@@ -37748,7 +37748,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>NOMURA HOLDINGS INC.</t>
+          <t>野村ホールディングス</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -37897,7 +37897,7 @@
         <v>1554</v>
       </c>
       <c r="AV4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW4" t="n">
         <v>0</v>
@@ -37933,7 +37933,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DAIICHI LIFE GROUP INC</t>
+          <t>第一生命ホールディングス</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -38086,7 +38086,7 @@
         <v>1841.5</v>
       </c>
       <c r="AV5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
@@ -38122,7 +38122,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DAIWA SECURITIES GROUP</t>
+          <t>大和証券グループ本社</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -38271,7 +38271,7 @@
         <v>1771</v>
       </c>
       <c r="AV6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW6" t="n">
         <v>0</v>
@@ -38307,7 +38307,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YOKOHAMA RUBBER CO</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -38456,7 +38456,7 @@
         <v>7647</v>
       </c>
       <c r="AV7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW7" t="n">
         <v>0</v>
@@ -38492,7 +38492,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>LY CORPORATION</t>
+          <t>LINEヤフー</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -38641,7 +38641,7 @@
         <v>497.9</v>
       </c>
       <c r="AV8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW8" t="n">
         <v>0</v>
@@ -38677,7 +38677,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DIC CORPORATION</t>
+          <t>DIC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -38826,7 +38826,7 @@
         <v>5495</v>
       </c>
       <c r="AV9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW9" t="n">
         <v>0</v>
@@ -38862,7 +38862,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MIZUHO FINANCIAL GROUP</t>
+          <t>みずほフィナンシャルグループ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -39015,7 +39015,7 @@
         <v>8531</v>
       </c>
       <c r="AV10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW10" t="n">
         <v>0</v>
@@ -39051,7 +39051,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">MITSUBISHI UFJ FINANCIAL GROUP </t>
+          <t>三菱UFJフィナンシャル・グループ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -39204,7 +39204,7 @@
         <v>3654</v>
       </c>
       <c r="AV11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW11" t="n">
         <v>0</v>
@@ -39240,7 +39240,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>CHIBA BANK</t>
+          <t>千葉銀行</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -39389,7 +39389,7 @@
         <v>2837.5</v>
       </c>
       <c r="AV12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW12" t="n">
         <v>0</v>
@@ -39425,7 +39425,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MS&amp;AD INS GP HLDGS</t>
+          <t>MS&amp;ADインシュアランスグループホールディングス</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -39574,7 +39574,7 @@
         <v>4985</v>
       </c>
       <c r="AV13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW13" t="n">
         <v>0</v>
@@ -39610,7 +39610,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KIRIN HOLDINGS COMPANY LIMITED</t>
+          <t>キリンホールディングス</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -39759,7 +39759,7 @@
         <v>3000</v>
       </c>
       <c r="AV14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW14" t="n">
         <v>0</v>
@@ -39795,7 +39795,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BRIDGESTONE CORP</t>
+          <t>ブリヂストン</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -39944,7 +39944,7 @@
         <v>4074</v>
       </c>
       <c r="AV15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW15" t="n">
         <v>0</v>
@@ -39980,7 +39980,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>NISSAN CHEMICAL CORPORATION</t>
+          <t>日産化学</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -40129,7 +40129,7 @@
         <v>8059</v>
       </c>
       <c r="AV16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW16" t="n">
         <v>0</v>
@@ -40165,7 +40165,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>IDEMITSU KOSAN CO.LTD</t>
+          <t>出光興産</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -40314,7 +40314,7 @@
         <v>1370.5</v>
       </c>
       <c r="AV17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW17" t="n">
         <v>0</v>
@@ -40350,7 +40350,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OTSUKA HLDGS CO LTD</t>
+          <t>大塚ホールディングス</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -40499,7 +40499,7 @@
         <v>12040</v>
       </c>
       <c r="AV18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW18" t="n">
         <v>0</v>
@@ -40535,7 +40535,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SUMITOMO MITSUI FINANCIAL GROUP</t>
+          <t>三井住友フィナンシャルグループ</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -40688,7 +40688,7 @@
         <v>6900</v>
       </c>
       <c r="AV19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW19" t="n">
         <v>0</v>
@@ -40724,7 +40724,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>NICHIREI CORP</t>
+          <t>ニチレイ</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -40873,7 +40873,7 @@
         <v>2141.5</v>
       </c>
       <c r="AV20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW20" t="n">
         <v>0</v>
@@ -41200,7 +41200,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ADVANTEST CORP</t>
+          <t>アドバンテスト</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -41371,7 +41371,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NITTO DENKO CORP</t>
+          <t>日東電工</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -41542,7 +41542,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SEIKO EPSON CORP</t>
+          <t>セイコーエプソン</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -41713,7 +41713,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SONY GROUP CORPORATION</t>
+          <t>ソニーグループ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -41884,7 +41884,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FUJI ELECTRIC CO. LTD.</t>
+          <t>富士電機</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -42055,7 +42055,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KEYENCE CORP</t>
+          <t>キーエンス</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -42224,7 +42224,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>NIDEC CORPORATION</t>
+          <t>ニデック</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -42395,7 +42395,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NEC CORP</t>
+          <t>NEC</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -42566,7 +42566,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SOFTBANK GROUP CORP</t>
+          <t>ソフトバンクグループ</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -42737,7 +42737,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MITSUBISHI ELECTRIC CORP</t>
+          <t>三菱電機</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -42906,7 +42906,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>HITACHI</t>
+          <t>日立製作所</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -43075,7 +43075,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TOKYO ELECTRON</t>
+          <t>東京エレクトロン</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -43246,7 +43246,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KIOXIA HOLDINGS CORPORATION</t>
+          <t>キオクシアホールディングス</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -43413,7 +43413,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MURATA MANUFACTURING CO</t>
+          <t>村田製作所</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -43584,7 +43584,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RENESAS ELECTRONICS CORP</t>
+          <t>ルネサスエレクトロニクス</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -43753,7 +43753,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FUJITSU</t>
+          <t>富士通</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -43924,7 +43924,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SHIN-ETSU CHEMICAL CO</t>
+          <t>信越化学工業</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -44386,7 +44386,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DAIICHI LIFE GROUP INC</t>
+          <t>第一生命ホールディングス</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -44539,7 +44539,7 @@
         <v>1841.5</v>
       </c>
       <c r="AV2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -44575,7 +44575,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>JAPAN TOBACCO INC</t>
+          <t>日本たばこ産業（JT）</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -44746,7 +44746,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SOFTBANK CORP.</t>
+          <t>ソフトバンク</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -44917,7 +44917,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>NTT INC</t>
+          <t>NTT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -45088,7 +45088,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TOKIO MARINE HOLDINGS INC</t>
+          <t>東京海上ホールディングス</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -45257,7 +45257,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>KDDI CORPORATION</t>
+          <t>KDDI</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -45428,7 +45428,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MITSUI &amp; CO</t>
+          <t>三井物産</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -45599,7 +45599,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SUMITOMO MITSUI TRUST GP INC</t>
+          <t>三井住友トラストグループ</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -45752,7 +45752,7 @@
         <v>1734</v>
       </c>
       <c r="AV9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW9" t="n">
         <v>0</v>
@@ -45788,7 +45788,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ORIX CORPORATION</t>
+          <t>オリックス</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -45959,7 +45959,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MITSUBISHI CORP</t>
+          <t>三菱商事</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -46130,7 +46130,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">MITSUBISHI UFJ FINANCIAL GROUP </t>
+          <t>三菱UFJフィナンシャル・グループ</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -46283,7 +46283,7 @@
         <v>3654</v>
       </c>
       <c r="AV12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW12" t="n">
         <v>0</v>
@@ -46319,7 +46319,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MARUBENI CORP</t>
+          <t>丸紅</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -46490,7 +46490,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ITOCHU CORP</t>
+          <t>伊藤忠商事</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -46661,7 +46661,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SUMITOMO MITSUI FINANCIAL GROUP</t>
+          <t>三井住友フィナンシャルグループ</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -46814,7 +46814,7 @@
         <v>6900</v>
       </c>
       <c r="AV15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW15" t="n">
         <v>0</v>
@@ -46850,7 +46850,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MIZUHO FINANCIAL GROUP</t>
+          <t>みずほフィナンシャルグループ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -47003,7 +47003,7 @@
         <v>8531</v>
       </c>
       <c r="AV16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW16" t="n">
         <v>0</v>
@@ -47039,7 +47039,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>RESONA HOLDINGS</t>
+          <t>りそなホールディングス</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -47501,7 +47501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SUMITOMO MITSUI TRUST GP INC</t>
+          <t>三井住友トラストグループ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -47654,7 +47654,7 @@
         <v>1734</v>
       </c>
       <c r="AV2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -47690,7 +47690,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SUZUKI MOTOR CORP</t>
+          <t>スズキ</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -47839,7 +47839,7 @@
         <v>2081</v>
       </c>
       <c r="AV3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW3" t="n">
         <v>0</v>
@@ -47875,7 +47875,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YOKOHAMA RUBBER CO</t>
+          <t>横浜ゴム</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -48024,7 +48024,7 @@
         <v>7647</v>
       </c>
       <c r="AV4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW4" t="n">
         <v>0</v>
@@ -48060,7 +48060,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MIZUHO FINANCIAL GROUP</t>
+          <t>みずほフィナンシャルグループ</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -48213,7 +48213,7 @@
         <v>8531</v>
       </c>
       <c r="AV5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
@@ -48249,7 +48249,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">MITSUBISHI UFJ FINANCIAL GROUP </t>
+          <t>三菱UFJフィナンシャル・グループ</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -48402,7 +48402,7 @@
         <v>3654</v>
       </c>
       <c r="AV6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW6" t="n">
         <v>0</v>
@@ -48438,7 +48438,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CHIBA BANK</t>
+          <t>千葉銀行</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -48587,7 +48587,7 @@
         <v>2837.5</v>
       </c>
       <c r="AV7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW7" t="n">
         <v>0</v>
@@ -48623,7 +48623,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MS&amp;AD INS GP HLDGS</t>
+          <t>MS&amp;ADインシュアランスグループホールディングス</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -48772,7 +48772,7 @@
         <v>4985</v>
       </c>
       <c r="AV8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW8" t="n">
         <v>0</v>
@@ -48808,7 +48808,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>NISSAN CHEMICAL CORPORATION</t>
+          <t>日産化学</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -48957,7 +48957,7 @@
         <v>8059</v>
       </c>
       <c r="AV9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW9" t="n">
         <v>0</v>
@@ -48993,7 +48993,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>IDEMITSU KOSAN CO.LTD</t>
+          <t>出光興産</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -49142,7 +49142,7 @@
         <v>1370.5</v>
       </c>
       <c r="AV10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW10" t="n">
         <v>0</v>
@@ -49178,7 +49178,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SUMITOMO MITSUI FINANCIAL GROUP</t>
+          <t>三井住友フィナンシャルグループ</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -49331,7 +49331,7 @@
         <v>6900</v>
       </c>
       <c r="AV11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW11" t="n">
         <v>0</v>
@@ -49658,7 +49658,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>NOMURA HOLDINGS INC.</t>
+          <t>野村ホールディングス</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -49807,7 +49807,7 @@
         <v>1554</v>
       </c>
       <c r="AV2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW2" t="n">
         <v>0</v>
@@ -49843,7 +49843,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DAIICHI LIFE GROUP INC</t>
+          <t>第一生命ホールディングス</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -49996,7 +49996,7 @@
         <v>1841.5</v>
       </c>
       <c r="AV3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW3" t="n">
         <v>0</v>
@@ -50032,7 +50032,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DAIWA SECURITIES GROUP</t>
+          <t>大和証券グループ本社</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -50181,7 +50181,7 @@
         <v>1771</v>
       </c>
       <c r="AV4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW4" t="n">
         <v>0</v>
@@ -50217,7 +50217,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LY CORPORATION</t>
+          <t>LINEヤフー</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -50366,7 +50366,7 @@
         <v>497.9</v>
       </c>
       <c r="AV5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW5" t="n">
         <v>0</v>
@@ -50402,7 +50402,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>KIRIN HOLDINGS COMPANY LIMITED</t>
+          <t>キリンホールディングス</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -50551,7 +50551,7 @@
         <v>3000</v>
       </c>
       <c r="AV6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AW6" t="n">
         <v>0</v>

</xml_diff>